<commit_message>
Frezyderm: prettified names + regenerated catalog
</commit_message>
<xml_diff>
--- a/frezyderm-catalog.xlsx
+++ b/frezyderm-catalog.xlsx
@@ -115,7 +115,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM  AQUA GEL LUBRICANT CARE  50GR</t>
+          <t xml:space="preserve">Frezyderm Aqua Gel Lubricant Care 50Gr</t>
         </is>
       </c>
       <c r="B2">
@@ -148,7 +148,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">BABY HYDRA MILK</t>
+          <t xml:space="preserve">Frezyderm Baby Hydra Milk</t>
         </is>
       </c>
       <c r="B3">
@@ -186,7 +186,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">BODY SHOWER REVITALIZING CLEANSER</t>
+          <t xml:space="preserve">Frezyderm Body Shower Revitalizing Cleanser</t>
         </is>
       </c>
       <c r="B4">
@@ -224,7 +224,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">CHRISTIALEN EMULSION</t>
+          <t xml:space="preserve">Frezyderm Christialen Emulsion</t>
         </is>
       </c>
       <c r="B5">
@@ -267,7 +267,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM  Elastin Refill Cream Booster 5ml</t>
+          <t xml:space="preserve">Frezyderm Elastin Refill Cream Booster 5ml</t>
         </is>
       </c>
       <c r="B6">
@@ -295,7 +295,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">NECK CONTOUR CREAM</t>
+          <t xml:space="preserve">Frezyderm Neck Contour Cream</t>
         </is>
       </c>
       <c r="B7">
@@ -333,7 +333,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">ABD REFORM SKIN TENSIONER CREAM GEL </t>
+          <t xml:space="preserve">Frezyderm Abd Reform Skin Tensioner Cream Gel</t>
         </is>
       </c>
       <c r="B8">
@@ -371,7 +371,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">AC-NORM ACTIVE CLEANSER</t>
+          <t xml:space="preserve">Frezyderm Ac-Norm Active Cleanser</t>
         </is>
       </c>
       <c r="B9">
@@ -409,7 +409,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">AC-NORM ACTIVE CLEANSER</t>
+          <t xml:space="preserve">Frezyderm Ac-Norm Active Cleanser</t>
         </is>
       </c>
       <c r="B10">
@@ -447,7 +447,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">AC-NORM ACTIVE FOAM PLUS </t>
+          <t xml:space="preserve">Frezyderm Ac-Norm Active Foam Plus</t>
         </is>
       </c>
       <c r="B11">
@@ -490,7 +490,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">AC-NORM ACTIVE FOAM PLUS </t>
+          <t xml:space="preserve">Frezyderm Ac-Norm Active Foam Plus</t>
         </is>
       </c>
       <c r="B12">
@@ -528,7 +528,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">AC-NORM AQUATIC SERUM</t>
+          <t xml:space="preserve">Frezyderm Ac-Norm Aquatic Serum</t>
         </is>
       </c>
       <c r="B13">
@@ -566,7 +566,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">AC-NORM AQUATIC SERUM</t>
+          <t xml:space="preserve">Frezyderm Ac-Norm Aquatic Serum</t>
         </is>
       </c>
       <c r="B14">
@@ -604,7 +604,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">AC-NORM AQUATIC SERUM</t>
+          <t xml:space="preserve">Frezyderm Ac-Norm Aquatic Serum</t>
         </is>
       </c>
       <c r="B15">
@@ -642,7 +642,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM AcNorm Baby Cream 40ml</t>
+          <t xml:space="preserve">Frezyderm AcNorm Baby Cream 40ml</t>
         </is>
       </c>
       <c r="B16">
@@ -670,7 +670,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">AC-NORM HYDRA SCREEN SPF 15</t>
+          <t xml:space="preserve">Frezyderm Ac-Norm Hydra Screen Spf 15</t>
         </is>
       </c>
       <c r="B17">
@@ -708,7 +708,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">AC-NORM LIP BALM SPF 15</t>
+          <t xml:space="preserve">Frezyderm Ac-Norm Lip Balm Spf 15</t>
         </is>
       </c>
       <c r="B18">
@@ -746,7 +746,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">AC-NORM MEDILIKE EFFECT 1 CREAM</t>
+          <t xml:space="preserve">Frezyderm Ac-Norm Medilike Effect 1 Cream</t>
         </is>
       </c>
       <c r="B19">
@@ -784,7 +784,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">AC-NORM MEDILIKE EFFECT 1 CREAM</t>
+          <t xml:space="preserve">Frezyderm Ac-Norm Medilike Effect 1 Cream</t>
         </is>
       </c>
       <c r="B20">
@@ -822,7 +822,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">AC-NORM MEDILIKE EFFECT 1 CREAM</t>
+          <t xml:space="preserve">Frezyderm Ac-Norm Medilike Effect 1 Cream</t>
         </is>
       </c>
       <c r="B21">
@@ -860,7 +860,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">AC-NORM MICELLAR WATER</t>
+          <t xml:space="preserve">Frezyderm Ac-Norm Micellar Water</t>
         </is>
       </c>
       <c r="B22">
@@ -898,7 +898,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">AC-NORM NORMALIZING LOTION</t>
+          <t xml:space="preserve">Frezyderm Ac-Norm Normalizing Lotion</t>
         </is>
       </c>
       <c r="B23">
@@ -936,7 +936,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">AC-NORM PEELING GEL</t>
+          <t xml:space="preserve">Frezyderm Ac-Norm Peeling Gel</t>
         </is>
       </c>
       <c r="B24">
@@ -974,7 +974,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">AC-NORM PEELING GEL</t>
+          <t xml:space="preserve">Frezyderm Ac-Norm Peeling Gel</t>
         </is>
       </c>
       <c r="B25">
@@ -1012,7 +1012,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">AC-NORM PEEL-OFF MASK</t>
+          <t xml:space="preserve">Frezyderm Ac-Norm Peel-Off Mask</t>
         </is>
       </c>
       <c r="B26">
@@ -1050,7 +1050,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">AC-NORM SEB ADSORB CREAM</t>
+          <t xml:space="preserve">Frezyderm Ac-Norm Seb Adsorb Cream</t>
         </is>
       </c>
       <c r="B27">
@@ -1088,7 +1088,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">AC-NORM SPOT CARE</t>
+          <t xml:space="preserve">Frezyderm Ac-Norm Spot Care</t>
         </is>
       </c>
       <c r="B28">
@@ -1126,7 +1126,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">AC-NORM SPOT CARE</t>
+          <t xml:space="preserve">Frezyderm Ac-Norm Spot Care</t>
         </is>
       </c>
       <c r="B29">
@@ -1164,7 +1164,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">AC-NORM SUN SCREEN FLUID ΜΑΤ SPF 50+</t>
+          <t xml:space="preserve">Frezyderm Ac-Norm Sun Screen Fluid ΜΑΤ Spf 50+</t>
         </is>
       </c>
       <c r="B30">
@@ -1202,7 +1202,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">AC-NORM SUN SCREEN FLUID TINTED ΜΑΤ SPF 50+</t>
+          <t xml:space="preserve">Frezyderm Ac-Norm Sun Screen Fluid Tinted ΜΑΤ Spf 50+</t>
         </is>
       </c>
       <c r="B31">
@@ -1240,7 +1240,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">AC-NORM ACTIVE FOAM PLUS </t>
+          <t xml:space="preserve">Frezyderm Ac-Norm Active Foam Plus</t>
         </is>
       </c>
       <c r="B32">
@@ -1278,7 +1278,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">AC-NORM TOTAL CONTROL CREAM</t>
+          <t xml:space="preserve">Frezyderm Ac-Norm Total Control Cream</t>
         </is>
       </c>
       <c r="B33">
@@ -1316,7 +1316,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">ACTIVE BLOCK SPF 25</t>
+          <t xml:space="preserve">Frezyderm Active Block Spf 25</t>
         </is>
       </c>
       <c r="B34">
@@ -1354,7 +1354,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM ACTIVE S.SCREEN TINDED F.CREAM Spf50+50ML</t>
+          <t xml:space="preserve">Frezyderm Active S.Screen Tinded F.Cream Spf50+50Ml</t>
         </is>
       </c>
       <c r="B35">
@@ -1387,7 +1387,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">ACTIVE SUN SCREEN FACE FOUNDATION SPF 30</t>
+          <t xml:space="preserve">Frezyderm Active Sun Screen Face Foundation Spf 30</t>
         </is>
       </c>
       <c r="B36">
@@ -1425,7 +1425,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">ACTIVE SUN SCREEN SENSITIVE FACE - BODY SPF 50</t>
+          <t xml:space="preserve">Frezyderm Active Sun Screen Sensitive Face - Body Spf 50</t>
         </is>
       </c>
       <c r="B37">
@@ -1463,7 +1463,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUN SCREEN VELVET FACE SPF 30 </t>
+          <t xml:space="preserve">Frezyderm Sun Screen Velvet Face Spf 30</t>
         </is>
       </c>
       <c r="B38">
@@ -1501,7 +1501,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">AC-NORM SUN SCREEN FLUID ΜΑΤ SPF 50+</t>
+          <t xml:space="preserve">Frezyderm Ac-Norm Sun Screen Fluid ΜΑΤ Spf 50+</t>
         </is>
       </c>
       <c r="B39">
@@ -1539,7 +1539,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">AC-NORM SUN SCREEN FLUID ΜΑΤ SPF 50+</t>
+          <t xml:space="preserve">Frezyderm Ac-Norm Sun Screen Fluid ΜΑΤ Spf 50+</t>
         </is>
       </c>
       <c r="B40">
@@ -1577,7 +1577,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">ACTIVE SUN SCREEN FACE FOUNDATION SPF 30</t>
+          <t xml:space="preserve">Frezyderm Active Sun Screen Face Foundation Spf 30</t>
         </is>
       </c>
       <c r="B41">
@@ -1615,7 +1615,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">ACTIVE SUN SCREEN LIP BALM SPF 50+</t>
+          <t xml:space="preserve">Frezyderm Active Sun Screen Lip Balm Spf 50+</t>
         </is>
       </c>
       <c r="B42">
@@ -1653,7 +1653,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">AC-NORM SUN SCREEN FLUID ΜΑΤ SPF 50+</t>
+          <t xml:space="preserve">Frezyderm Ac-Norm Sun Screen Fluid ΜΑΤ Spf 50+</t>
         </is>
       </c>
       <c r="B43">
@@ -1691,7 +1691,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUN SCREEN MOUSSE SPF 30</t>
+          <t xml:space="preserve">Frezyderm Sun Screen Mousse Spf 30</t>
         </is>
       </c>
       <c r="B44">
@@ -1729,7 +1729,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">AGE REPAIR SET</t>
+          <t xml:space="preserve">Frezyderm Age Repair Set</t>
         </is>
       </c>
       <c r="B45">
@@ -1767,7 +1767,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM Anti - Age Shampoo 200ml</t>
+          <t xml:space="preserve">Frezyderm Anti - Age Shampoo 200ml</t>
         </is>
       </c>
       <c r="B46">
@@ -1795,7 +1795,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve">ANTI-AGEING BODY CREAM</t>
+          <t xml:space="preserve">Frezyderm Anti-Ageing Body Cream</t>
         </is>
       </c>
       <c r="B47">
@@ -1833,7 +1833,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">ANTI-THERMAL SPRING SEA WATER MIST</t>
+          <t xml:space="preserve">Frezyderm Anti-Thermal Spring Sea Water Mist</t>
         </is>
       </c>
       <c r="B48">
@@ -1871,7 +1871,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM ANTICORT CREAM 50ml</t>
+          <t xml:space="preserve">Frezyderm Anticort Cream 50ml</t>
         </is>
       </c>
       <c r="B49">
@@ -1904,7 +1904,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve">ANTICORT OINTMENT</t>
+          <t xml:space="preserve">Frezyderm Anticort Ointment</t>
         </is>
       </c>
       <c r="B50">
@@ -1942,7 +1942,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM Antidandruff Shampoo 125ml</t>
+          <t xml:space="preserve">Frezyderm Antidandruff Shampoo 125ml</t>
         </is>
       </c>
       <c r="B51">
@@ -1975,7 +1975,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM ANTIDANDRUFF SHAMPOO SEBO 200ML</t>
+          <t xml:space="preserve">Frezyderm Antidandruff Shampoo Sebo 200Ml</t>
         </is>
       </c>
       <c r="B52">
@@ -2003,7 +2003,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">ANTIOXIDANT RADIATION GUARD SPF 50+</t>
+          <t xml:space="preserve">Frezyderm Antioxidant Radiation Guard Spf 50+</t>
         </is>
       </c>
       <c r="B53">
@@ -2041,7 +2041,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM Antioxidant Vitamin C Cream Booster 5ml</t>
+          <t xml:space="preserve">Frezyderm Antioxidant Vitamin C Cream Booster 5ml</t>
         </is>
       </c>
       <c r="B54">
@@ -2069,7 +2069,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM Antispot Cream Booster 5ml</t>
+          <t xml:space="preserve">Frezyderm Antispot Cream Booster 5ml</t>
         </is>
       </c>
       <c r="B55">
@@ -2097,7 +2097,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t xml:space="preserve">ANTI-WRINKLE RICH DAY CREAM</t>
+          <t xml:space="preserve">Frezyderm Anti-Wrinkle Rich Day Cream</t>
         </is>
       </c>
       <c r="B56">
@@ -2135,7 +2135,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t xml:space="preserve">ANTI-WRINKLE RICH DAY CREAM</t>
+          <t xml:space="preserve">Frezyderm Anti-Wrinkle Rich Day Cream</t>
         </is>
       </c>
       <c r="B57">
@@ -2173,7 +2173,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t xml:space="preserve">ANTI-WRINKLE RICH DAY CREAM</t>
+          <t xml:space="preserve">Frezyderm Anti-Wrinkle Rich Day Cream</t>
         </is>
       </c>
       <c r="B58">
@@ -2211,7 +2211,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t xml:space="preserve">APHTHAE GEL Adults  </t>
+          <t xml:space="preserve">Frezyderm Aphthae Gel Adults</t>
         </is>
       </c>
       <c r="B59">
@@ -2249,7 +2249,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM AQUA CARE  VAGINAL CREAM 50ML</t>
+          <t xml:space="preserve">Frezyderm Aqua Care Vaginal Cream 50Ml</t>
         </is>
       </c>
       <c r="B60">
@@ -2282,7 +2282,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t xml:space="preserve">BABY LAUNDRY</t>
+          <t xml:space="preserve">Frezyderm Baby Laundry</t>
         </is>
       </c>
       <c r="B61">
@@ -2325,7 +2325,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t xml:space="preserve">ATOPREL BARRIER CREAM</t>
+          <t xml:space="preserve">Frezyderm Atoprel Barrier Cream</t>
         </is>
       </c>
       <c r="B62">
@@ -2368,7 +2368,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t xml:space="preserve">ATOPREL MILKY BATH OIL</t>
+          <t xml:space="preserve">Frezyderm Atoprel Milky Bath Oil</t>
         </is>
       </c>
       <c r="B63">
@@ -2406,7 +2406,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t xml:space="preserve">ATOPREL MILKY BATH OIL</t>
+          <t xml:space="preserve">Frezyderm Atoprel Milky Bath Oil</t>
         </is>
       </c>
       <c r="B64">
@@ -2444,7 +2444,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t xml:space="preserve">ATOPREL EMOLLIENT BAUME</t>
+          <t xml:space="preserve">Frezyderm Atoprel Emollient Baume</t>
         </is>
       </c>
       <c r="B65">
@@ -2482,7 +2482,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t xml:space="preserve">ATOPREL EMOLLIENT CLASSIC</t>
+          <t xml:space="preserve">Frezyderm Atoprel Emollient Classic</t>
         </is>
       </c>
       <c r="B66">
@@ -2520,7 +2520,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t xml:space="preserve">ATOPREL EMOLLIENT BAUME</t>
+          <t xml:space="preserve">Frezyderm Atoprel Emollient Baume</t>
         </is>
       </c>
       <c r="B67">
@@ -2558,7 +2558,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t xml:space="preserve">ATOPREL EMOLLIENT MOUSSE</t>
+          <t xml:space="preserve">Frezyderm Atoprel Emollient Mousse</t>
         </is>
       </c>
       <c r="B68">
@@ -2596,7 +2596,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t xml:space="preserve">ATOPREL FOAMY SHAMPOO</t>
+          <t xml:space="preserve">Frezyderm Atoprel Foamy Shampoo</t>
         </is>
       </c>
       <c r="B69">
@@ -2634,7 +2634,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t xml:space="preserve">ATOPREL FOAMY SHAMPOO</t>
+          <t xml:space="preserve">Frezyderm Atoprel Foamy Shampoo</t>
         </is>
       </c>
       <c r="B70">
@@ -2672,7 +2672,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t xml:space="preserve">ATOPREL MILKY BATH OIL</t>
+          <t xml:space="preserve">Frezyderm Atoprel Milky Bath Oil</t>
         </is>
       </c>
       <c r="B71">
@@ -2710,7 +2710,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM BABY ABCC 50ML</t>
+          <t xml:space="preserve">Frezyderm Baby Abcc 50Ml</t>
         </is>
       </c>
       <c r="B72">
@@ -2743,7 +2743,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t xml:space="preserve">BABY BATH</t>
+          <t xml:space="preserve">Frezyderm Baby Bath</t>
         </is>
       </c>
       <c r="B73">
@@ -2781,7 +2781,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t xml:space="preserve">BABY BATH</t>
+          <t xml:space="preserve">Frezyderm Baby Bath</t>
         </is>
       </c>
       <c r="B74">
@@ -2819,7 +2819,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t xml:space="preserve">BABY CHAMOMILE BATH</t>
+          <t xml:space="preserve">Frezyderm Baby Chamomile Bath</t>
         </is>
       </c>
       <c r="B75">
@@ -2857,7 +2857,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t xml:space="preserve">BABY COLOGNE</t>
+          <t xml:space="preserve">Frezyderm Baby Cologne</t>
         </is>
       </c>
       <c r="B76">
@@ -2895,7 +2895,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM BABY CREAM  175 ml</t>
+          <t xml:space="preserve">Frezyderm Baby Cream 175 ml</t>
         </is>
       </c>
       <c r="B77">
@@ -2928,7 +2928,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM Baby Cream 50ml</t>
+          <t xml:space="preserve">Frezyderm Baby Cream 50ml</t>
         </is>
       </c>
       <c r="B78">
@@ -2961,7 +2961,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM BABY FOAM 150ML</t>
+          <t xml:space="preserve">Frezyderm Baby Foam 150Ml</t>
         </is>
       </c>
       <c r="B79">
@@ -2989,7 +2989,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t xml:space="preserve">BABY GUMS GEL</t>
+          <t xml:space="preserve">Frezyderm Baby Gums Gel</t>
         </is>
       </c>
       <c r="B80">
@@ -3027,7 +3027,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t xml:space="preserve">BABY HYDRA MILK</t>
+          <t xml:space="preserve">Frezyderm Baby Hydra Milk</t>
         </is>
       </c>
       <c r="B81">
@@ -3065,7 +3065,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t xml:space="preserve">BABY LIQUID TALC</t>
+          <t xml:space="preserve">Frezyderm Baby Liquid Talc</t>
         </is>
       </c>
       <c r="B82">
@@ -3103,7 +3103,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t xml:space="preserve">BABY OIL</t>
+          <t xml:space="preserve">Frezyderm Baby Oil</t>
         </is>
       </c>
       <c r="B83">
@@ -3141,7 +3141,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t xml:space="preserve">BABY PERIORAL ΟΙΝΤΜΕΝΤ</t>
+          <t xml:space="preserve">Frezyderm Baby Perioral ΟΙΝΤΜΕΝΤ</t>
         </is>
       </c>
       <c r="B84">
@@ -3179,7 +3179,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t xml:space="preserve">BABY PERIORAL ΟΙΝΤΜΕΝΤ</t>
+          <t xml:space="preserve">Frezyderm Baby Perioral ΟΙΝΤΜΕΝΤ</t>
         </is>
       </c>
       <c r="B85">
@@ -3217,7 +3217,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM Baby Shampoo 200ml</t>
+          <t xml:space="preserve">Frezyderm Baby Shampoo 200ml</t>
         </is>
       </c>
       <c r="B86">
@@ -3245,7 +3245,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM BABY SHAMPOO 300ML</t>
+          <t xml:space="preserve">Frezyderm Baby Shampoo 300Ml</t>
         </is>
       </c>
       <c r="B87">
@@ -3273,7 +3273,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t xml:space="preserve">BABY SUN CARE SPF 25</t>
+          <t xml:space="preserve">Frezyderm Baby Sun Care Spf 25</t>
         </is>
       </c>
       <c r="B88">
@@ -3311,7 +3311,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t xml:space="preserve">BABY SUN CARE SPF 25</t>
+          <t xml:space="preserve">Frezyderm Baby Sun Care Spf 25</t>
         </is>
       </c>
       <c r="B89">
@@ -3349,7 +3349,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t xml:space="preserve">ANTI-THERMAL SPRING SEA WATER MIST</t>
+          <t xml:space="preserve">Frezyderm Anti-Thermal Spring Sea Water Mist</t>
         </is>
       </c>
       <c r="B90">
@@ -3387,7 +3387,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM CHLORHEXENE GEL 30ML</t>
+          <t xml:space="preserve">Frezyderm Chlorhexene Gel 30Ml</t>
         </is>
       </c>
       <c r="B91">
@@ -3415,7 +3415,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t xml:space="preserve">CHLORHEXENE PRO MOUTHWASH</t>
+          <t xml:space="preserve">Frezyderm Chlorhexene Pro Mouthwash</t>
         </is>
       </c>
       <c r="B92">
@@ -3453,7 +3453,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t xml:space="preserve">CHRISTIALEN EMULSION</t>
+          <t xml:space="preserve">Frezyderm Christialen Emulsion</t>
         </is>
       </c>
       <c r="B93">
@@ -3491,7 +3491,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYMAR CLEANER HYPERTONIC STRONG </t>
+          <t xml:space="preserve">Frezyderm Frezymar Cleaner Hypertonic Strong</t>
         </is>
       </c>
       <c r="B94">
@@ -3529,7 +3529,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t xml:space="preserve">BABY COLI SLEEP MASSAGE GEL</t>
+          <t xml:space="preserve">Frezyderm Baby Coli Sleep Massage Gel</t>
         </is>
       </c>
       <c r="B95">
@@ -3572,7 +3572,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t xml:space="preserve">COLOR EYE BALM</t>
+          <t xml:space="preserve">Frezyderm Color Eye Balm</t>
         </is>
       </c>
       <c r="B96">
@@ -3615,7 +3615,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM Color Protect Shampoo 200ml</t>
+          <t xml:space="preserve">Frezyderm Color Protect Shampoo 200ml</t>
         </is>
       </c>
       <c r="B97">
@@ -3643,7 +3643,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM Color Protect Spray 100ml</t>
+          <t xml:space="preserve">Frezyderm Color Protect Spray 100ml</t>
         </is>
       </c>
       <c r="B98">
@@ -3676,7 +3676,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t xml:space="preserve">UP CONFIDENCE BUST RECOVERY CREAM GEL</t>
+          <t xml:space="preserve">Frezyderm Up Confidence Bust Recovery Cream Gel</t>
         </is>
       </c>
       <c r="B99">
@@ -3714,7 +3714,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t xml:space="preserve">COUGH SYRUP ADULTS</t>
+          <t xml:space="preserve">Frezyderm Cough Syrup Adults</t>
         </is>
       </c>
       <c r="B100">
@@ -3752,7 +3752,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t xml:space="preserve">COUGH SYRUP KIDS</t>
+          <t xml:space="preserve">Frezyderm Cough Syrup Kids</t>
         </is>
       </c>
       <c r="B101">
@@ -3790,7 +3790,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t xml:space="preserve">CRILEN ANTI-MOSQUITO 10%</t>
+          <t xml:space="preserve">Frezyderm Crilen Anti-Mosquito 10%</t>
         </is>
       </c>
       <c r="B102">
@@ -3828,7 +3828,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t xml:space="preserve">CRILEN ANTI-MOSQUITO PLUS SPRAY 20%</t>
+          <t xml:space="preserve">Frezyderm Crilen Anti-Mosquito Plus Spray 20%</t>
         </is>
       </c>
       <c r="B103">
@@ -3866,7 +3866,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t xml:space="preserve">CRILEN ΓΑΛΑΚΤΩΜΑ 125ml ΜΕ ΔΩΡΟ ΕΠΙΠΛΕΟΝ ΠΟΣΟΤΗΤΑ 40ml</t>
+          <t xml:space="preserve">Frezyderm Crilen ΓΑΛΑΚΤΩΜΑ 125ml ΜΕ ΔΩΡΟ ΕΠΙΠΛΕΟΝ ΠΟΣΟΤΗΤΑ 40ml</t>
         </is>
       </c>
       <c r="B104">
@@ -3904,7 +3904,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t xml:space="preserve">CRILEN ADULT PLUS</t>
+          <t xml:space="preserve">Frezyderm Crilen Adult Plus</t>
         </is>
       </c>
       <c r="B105">
@@ -3942,7 +3942,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t xml:space="preserve">CRILEN AFTER NIP Gel</t>
+          <t xml:space="preserve">Frezyderm Crilen After Nip Gel</t>
         </is>
       </c>
       <c r="B106">
@@ -3985,7 +3985,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM Crilen Cream 50ml</t>
+          <t xml:space="preserve">Frezyderm Crilen Cream 50ml</t>
         </is>
       </c>
       <c r="B107">
@@ -4018,7 +4018,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t xml:space="preserve">CRILEN MOUSSE</t>
+          <t xml:space="preserve">Frezyderm Crilen Mousse</t>
         </is>
       </c>
       <c r="B108">
@@ -4056,7 +4056,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t xml:space="preserve">CRILEN ROLL BALL</t>
+          <t xml:space="preserve">Frezyderm Crilen Roll Ball</t>
         </is>
       </c>
       <c r="B109">
@@ -4094,7 +4094,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t xml:space="preserve">CRILEN ANTI-MOSQUITO PLUS SPRAY 20%</t>
+          <t xml:space="preserve">Frezyderm Crilen Anti-Mosquito Plus Spray 20%</t>
         </is>
       </c>
       <c r="B110">
@@ -4137,7 +4137,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t xml:space="preserve">DE-MAKE UP 4 in 1</t>
+          <t xml:space="preserve">Frezyderm De-Make Up 4 in 1</t>
         </is>
       </c>
       <c r="B111">
@@ -4175,7 +4175,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM Dermiox Cream 50ml</t>
+          <t xml:space="preserve">Frezyderm Dermiox Cream 50ml</t>
         </is>
       </c>
       <c r="B112">
@@ -4213,7 +4213,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t xml:space="preserve">DERMOFILIA ADULTS DEO CREAM</t>
+          <t xml:space="preserve">Frezyderm Dermofilia Adults Deo Cream</t>
         </is>
       </c>
       <c r="B113">
@@ -4251,7 +4251,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t xml:space="preserve">DERMOFILIA HAND CREAM 75ml ΜΕ ΔΩΡΟ ΕΠΙΠΛΕΟΝ ΠΟΣΟΤΗΤΑ 40ml</t>
+          <t xml:space="preserve">Frezyderm Dermofilia Hand Cream 75ml ΜΕ ΔΩΡΟ ΕΠΙΠΛΕΟΝ ΠΟΣΟΤΗΤΑ 40ml</t>
         </is>
       </c>
       <c r="B114">
@@ -4289,7 +4289,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t xml:space="preserve">DERMOFILIA HAND CREAM 75ml ΜΕ ΔΩΡΟ ΕΠΙΠΛΕΟΝ ΠΟΣΟΤΗΤΑ 40ml</t>
+          <t xml:space="preserve">Frezyderm Dermofilia Hand Cream 75ml ΜΕ ΔΩΡΟ ΕΠΙΠΛΕΟΝ ΠΟΣΟΤΗΤΑ 40ml</t>
         </is>
       </c>
       <c r="B115">
@@ -4332,7 +4332,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t xml:space="preserve">DIABETEETH TOOTHPASTE</t>
+          <t xml:space="preserve">Frezyderm Diabeteeth Toothpaste</t>
         </is>
       </c>
       <c r="B116">
@@ -4370,7 +4370,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t xml:space="preserve">DIAMOND VELVET ΑΝΤΙ-WRINKLE CREAM</t>
+          <t xml:space="preserve">Frezyderm Diamond Velvet ΑΝΤΙ-Wrinkle Cream</t>
         </is>
       </c>
       <c r="B117">
@@ -4408,7 +4408,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t xml:space="preserve">DIAMOND VELVET MOISTURIZING CREAM</t>
+          <t xml:space="preserve">Frezyderm Diamond Velvet Moisturizing Cream</t>
         </is>
       </c>
       <c r="B118">
@@ -4446,7 +4446,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM DMANNOSA 14 sachets 4gr</t>
+          <t xml:space="preserve">Frezyderm Dmannosa 14 sachets 4gr</t>
         </is>
       </c>
       <c r="B119">
@@ -4474,7 +4474,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM Ecovag Balance Κολπικά Υπόθετα για Αποκατάσταση της Κολπικής Χλωρίδας 10τμχ</t>
+          <t xml:space="preserve">Frezyderm Ecovag Balance Κολπικά Υπόθετα για Αποκατάσταση της Κολπικής Χλωρίδας 10τμχ</t>
         </is>
       </c>
       <c r="B120">
@@ -4502,7 +4502,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM EVERY DAY SHAMPOO 200ML</t>
+          <t xml:space="preserve">Frezyderm Every Day Shampoo 200Ml</t>
         </is>
       </c>
       <c r="B121">
@@ -4535,7 +4535,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM Expression Blocker Cream Booster 5ml</t>
+          <t xml:space="preserve">Frezyderm Expression Blocker Cream Booster 5ml</t>
         </is>
       </c>
       <c r="B122">
@@ -4563,7 +4563,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t xml:space="preserve">AC-NORM LIP BALM SPF 15</t>
+          <t xml:space="preserve">Frezyderm Ac-Norm Lip Balm Spf 15</t>
         </is>
       </c>
       <c r="B123">
@@ -4601,7 +4601,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM Face Tightener Cream Booster 5ml</t>
+          <t xml:space="preserve">Frezyderm Face Tightener Cream Booster 5ml</t>
         </is>
       </c>
       <c r="B124">
@@ -4634,7 +4634,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM Facial Scrub 100ml</t>
+          <t xml:space="preserve">Frezyderm Facial Scrub 100ml</t>
         </is>
       </c>
       <c r="B125">
@@ -4667,7 +4667,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM FERTI BOX OF 30 SACHETS OF 2,5</t>
+          <t xml:space="preserve">Frezyderm Ferti Box Of 30 Sachets Of 2,5</t>
         </is>
       </c>
       <c r="B126">
@@ -4695,7 +4695,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t xml:space="preserve">FIRST AID BUTTER</t>
+          <t xml:space="preserve">Frezyderm First Aid Butter</t>
         </is>
       </c>
       <c r="B127">
@@ -4733,7 +4733,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t xml:space="preserve">PRODILAC IMMUNO SHIELD FAST MELT</t>
+          <t xml:space="preserve">Frezyderm Prodilac Immuno Shield Fast Melt</t>
         </is>
       </c>
       <c r="B128">
@@ -4771,7 +4771,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM Frezyderm Promo Νεσεσέρ με Moisturizing Rich Cream 50ml &amp; Super Booster 5ml -30%</t>
+          <t xml:space="preserve">Frezyderm Frezyderm Promo Νεσεσέρ με Moisturizing Rich Cream 50ml &amp; Super Booster 5ml -30%</t>
         </is>
       </c>
       <c r="B129">
@@ -4804,7 +4804,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYFEET DIAPED CREAM</t>
+          <t xml:space="preserve">Frezyderm Frezyfeet Diaped Cream</t>
         </is>
       </c>
       <c r="B130">
@@ -4842,7 +4842,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYFEET HEAVY LEGS</t>
+          <t xml:space="preserve">Frezyderm Frezyfeet Heavy Legs</t>
         </is>
       </c>
       <c r="B131">
@@ -4880,7 +4880,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYFEET KERACTIVE CREAM</t>
+          <t xml:space="preserve">Frezyderm Frezyfeet Keractive Cream</t>
         </is>
       </c>
       <c r="B132">
@@ -4918,7 +4918,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYFEET ODOR STOP SPRAY</t>
+          <t xml:space="preserve">Frezyderm Frezyfeet Odor Stop Spray</t>
         </is>
       </c>
       <c r="B133">
@@ -4956,7 +4956,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYFEET REVITAL CREAM</t>
+          <t xml:space="preserve">Frezyderm Frezyfeet Revital Cream</t>
         </is>
       </c>
       <c r="B134">
@@ -4994,7 +4994,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM FREZYKELD CREAM 40ML</t>
+          <t xml:space="preserve">Frezyderm Frezykeld Cream 40Ml</t>
         </is>
       </c>
       <c r="B135">
@@ -5022,7 +5022,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM Frezymar Baby Spray 100ml</t>
+          <t xml:space="preserve">Frezyderm Frezymar Baby Spray 100ml</t>
         </is>
       </c>
       <c r="B136">
@@ -5060,7 +5060,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYMAR CLEANER HYPERTONIC ALOE &amp; EUCALYPTUS MEDIUM</t>
+          <t xml:space="preserve">Frezyderm Frezymar Cleaner Hypertonic Aloe &amp; Eucalyptus Medium</t>
         </is>
       </c>
       <c r="B137">
@@ -5098,7 +5098,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYMAR CLEANER HYPERTONIC SOFT</t>
+          <t xml:space="preserve">Frezyderm Frezymar Cleaner Hypertonic Soft</t>
         </is>
       </c>
       <c r="B138">
@@ -5136,7 +5136,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM Frezymar Normal Spray 100ml</t>
+          <t xml:space="preserve">Frezyderm Frezymar Normal Spray 100ml</t>
         </is>
       </c>
       <c r="B139">
@@ -5174,7 +5174,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM Hair Balance Shampoo 200ml</t>
+          <t xml:space="preserve">Frezyderm Hair Balance Shampoo 200ml</t>
         </is>
       </c>
       <c r="B140">
@@ -5202,7 +5202,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t xml:space="preserve">HAIR FORCE SHAMPOO MEN</t>
+          <t xml:space="preserve">Frezyderm Hair Force Shampoo Men</t>
         </is>
       </c>
       <c r="B141">
@@ -5240,7 +5240,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t xml:space="preserve">HAIR FORCE SHAMPOO MEN</t>
+          <t xml:space="preserve">Frezyderm Hair Force Shampoo Men</t>
         </is>
       </c>
       <c r="B142">
@@ -5278,7 +5278,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t xml:space="preserve">HAIR FORCE SHAMPOO MEN</t>
+          <t xml:space="preserve">Frezyderm Hair Force Shampoo Men</t>
         </is>
       </c>
       <c r="B143">
@@ -5316,7 +5316,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t xml:space="preserve">HAIR FORCE SHAMPOO MEN</t>
+          <t xml:space="preserve">Frezyderm Hair Force Shampoo Men</t>
         </is>
       </c>
       <c r="B144">
@@ -5354,7 +5354,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t xml:space="preserve">HAIR FORCE SHAMPOO WOMEN</t>
+          <t xml:space="preserve">Frezyderm Hair Force Shampoo Women</t>
         </is>
       </c>
       <c r="B145">
@@ -5392,7 +5392,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t xml:space="preserve">HAIR FORCE TABS</t>
+          <t xml:space="preserve">Frezyderm Hair Force Tabs</t>
         </is>
       </c>
       <c r="B146">
@@ -5430,7 +5430,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t xml:space="preserve">HAIR FORCE SHAMPOO MEN</t>
+          <t xml:space="preserve">Frezyderm Hair Force Shampoo Men</t>
         </is>
       </c>
       <c r="B147">
@@ -5473,7 +5473,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM Hair Implant Shampoo 150ml</t>
+          <t xml:space="preserve">Frezyderm Hair Implant Shampoo 150ml</t>
         </is>
       </c>
       <c r="B148">
@@ -5501,7 +5501,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM Hair Repair Conditioner 200ml</t>
+          <t xml:space="preserve">Frezyderm Hair Repair Conditioner 200ml</t>
         </is>
       </c>
       <c r="B149">
@@ -5529,7 +5529,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM Hair Repair Mask 200ml</t>
+          <t xml:space="preserve">Frezyderm Hair Repair Mask 200ml</t>
         </is>
       </c>
       <c r="B150">
@@ -5562,7 +5562,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM Hair Repair Shampoo 200ml</t>
+          <t xml:space="preserve">Frezyderm Hair Repair Shampoo 200ml</t>
         </is>
       </c>
       <c r="B151">
@@ -5590,7 +5590,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM HOLISTIC ARNICA CREAM 100 ML</t>
+          <t xml:space="preserve">Frezyderm Holistic Arnica Cream 100 Ml</t>
         </is>
       </c>
       <c r="B152">
@@ -5623,7 +5623,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM HOLISTIC ARNICA CREAM 50ML</t>
+          <t xml:space="preserve">Frezyderm Holistic Arnica Cream 50Ml</t>
         </is>
       </c>
       <c r="B153">
@@ -5656,7 +5656,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM Holistic Calendula Cream 50ml</t>
+          <t xml:space="preserve">Frezyderm Holistic Calendula Cream 50ml</t>
         </is>
       </c>
       <c r="B154">
@@ -5689,7 +5689,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM Holistic Hypericum Cream 50ml</t>
+          <t xml:space="preserve">Frezyderm Holistic Hypericum Cream 50ml</t>
         </is>
       </c>
       <c r="B155">
@@ -5722,7 +5722,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM Holistic Propolis Cream 50ml</t>
+          <t xml:space="preserve">Frezyderm Holistic Propolis Cream 50ml</t>
         </is>
       </c>
       <c r="B156">
@@ -5755,7 +5755,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t xml:space="preserve">FACE SERUM HYALURONIC ACID - Ορός Ενυδάτωσης Προσώπου</t>
+          <t xml:space="preserve">Frezyderm Face Serum Hyaluronic Acid - Ορός Ενυδάτωσης Προσώπου</t>
         </is>
       </c>
       <c r="B157">
@@ -5793,7 +5793,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t xml:space="preserve">HYDRORAL XERO TOOTHPASTE</t>
+          <t xml:space="preserve">Frezyderm Hydroral Xero Toothpaste</t>
         </is>
       </c>
       <c r="B158">
@@ -5831,7 +5831,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t xml:space="preserve">HYDRORAL XERO MOUTHWASH </t>
+          <t xml:space="preserve">Frezyderm Hydroral Xero Mouthwash</t>
         </is>
       </c>
       <c r="B159">
@@ -5869,7 +5869,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t xml:space="preserve">HYDRORAL XERO TOOTHPASTE</t>
+          <t xml:space="preserve">Frezyderm Hydroral Xero Toothpaste</t>
         </is>
       </c>
       <c r="B160">
@@ -5907,7 +5907,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t xml:space="preserve">ICE EYES STICK </t>
+          <t xml:space="preserve">Frezyderm Ice Eyes Stick</t>
         </is>
       </c>
       <c r="B161">
@@ -5945,7 +5945,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM ICY  AFTER SUN  200ML</t>
+          <t xml:space="preserve">Frezyderm Icy After Sun 200Ml</t>
         </is>
       </c>
       <c r="B162">
@@ -5978,7 +5978,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t xml:space="preserve">INTIM VAGINAL DOUCHE MONODOSE ΞΥΔΙ pH 3.5</t>
+          <t xml:space="preserve">Frezyderm Intim Vaginal Douche Monodose ΞΥΔΙ pH 3.5</t>
         </is>
       </c>
       <c r="B163">
@@ -6016,7 +6016,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM IMMUNO (30caps*10)</t>
+          <t xml:space="preserve">Frezyderm Immuno (30caps*10)</t>
         </is>
       </c>
       <c r="B164">
@@ -6044,7 +6044,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t xml:space="preserve">INFANT SUN CARE SPF 50+</t>
+          <t xml:space="preserve">Frezyderm Infant Sun Care Spf 50+</t>
         </is>
       </c>
       <c r="B165">
@@ -6082,7 +6082,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM INSTANT LIFTING SERUM 15ML</t>
+          <t xml:space="preserve">Frezyderm Instant Lifting Serum 15Ml</t>
         </is>
       </c>
       <c r="B166">
@@ -6120,7 +6120,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t xml:space="preserve">INTIM AID CLEANSER</t>
+          <t xml:space="preserve">Frezyderm Intim Aid Cleanser</t>
         </is>
       </c>
       <c r="B167">
@@ -6158,7 +6158,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t xml:space="preserve">INTIM AID CLEANSER</t>
+          <t xml:space="preserve">Frezyderm Intim Aid Cleanser</t>
         </is>
       </c>
       <c r="B168">
@@ -6196,7 +6196,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t xml:space="preserve">INTIM AID CRANBERRY FOAM</t>
+          <t xml:space="preserve">Frezyderm Intim Aid Cranberry Foam</t>
         </is>
       </c>
       <c r="B169">
@@ -6234,7 +6234,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t xml:space="preserve">INTIM VAGINAL DOUCHE MONODOSE ΣΟΔΑ pH 9</t>
+          <t xml:space="preserve">Frezyderm Intim Vaginal Douche Monodose ΣΟΔΑ pH 9</t>
         </is>
       </c>
       <c r="B170">
@@ -6272,7 +6272,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t xml:space="preserve">INTIM AREA MENOPAUSE FOAM</t>
+          <t xml:space="preserve">Frezyderm Intim Area Menopause Foam</t>
         </is>
       </c>
       <c r="B171">
@@ -6315,7 +6315,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t xml:space="preserve">INTIM AREA MENOPAUSE FOAM</t>
+          <t xml:space="preserve">Frezyderm Intim Area Menopause Foam</t>
         </is>
       </c>
       <c r="B172">
@@ -6353,7 +6353,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t xml:space="preserve">INTIM AREA LIQUID </t>
+          <t xml:space="preserve">Frezyderm Intim Area Liquid</t>
         </is>
       </c>
       <c r="B173">
@@ -6391,7 +6391,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t xml:space="preserve">INTIM AREA LIQUID </t>
+          <t xml:space="preserve">Frezyderm Intim Area Liquid</t>
         </is>
       </c>
       <c r="B174">
@@ -6429,7 +6429,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t xml:space="preserve">INTIM AREA WIPES</t>
+          <t xml:space="preserve">Frezyderm Intim Area Wipes</t>
         </is>
       </c>
       <c r="B175">
@@ -6472,7 +6472,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t xml:space="preserve">INTIM VAGINAL DOUCHE MONODOSE ΣΟΔΑ pH 9</t>
+          <t xml:space="preserve">Frezyderm Intim Vaginal Douche Monodose ΣΟΔΑ pH 9</t>
         </is>
       </c>
       <c r="B176">
@@ -6510,7 +6510,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t xml:space="preserve">INTIM VAGINAL DOUCHE MONODOSE ΧΑΜΟΜΗΛΙ pH 4.5 </t>
+          <t xml:space="preserve">Frezyderm Intim Vaginal Douche Monodose ΧΑΜΟΜΗΛΙ pH 4.5</t>
         </is>
       </c>
       <c r="B177">
@@ -6548,7 +6548,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t xml:space="preserve">INTIM AID CLEANSER</t>
+          <t xml:space="preserve">Frezyderm Intim Aid Cleanser</t>
         </is>
       </c>
       <c r="B178">
@@ -6586,7 +6586,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM INTIMEO 14capsule</t>
+          <t xml:space="preserve">Frezyderm Intimeo 14capsule</t>
         </is>
       </c>
       <c r="B179">
@@ -6614,7 +6614,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM KIDS S.CARE CR SPRAY SPF50+275ML</t>
+          <t xml:space="preserve">Frezyderm Kids S.Care Cr Spray Spf50+275Ml</t>
         </is>
       </c>
       <c r="B180">
@@ -6647,7 +6647,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t xml:space="preserve">SENSITIVE KIDS DEODORANT CREAM</t>
+          <t xml:space="preserve">Frezyderm Sensitive Kids Deodorant Cream</t>
         </is>
       </c>
       <c r="B181">
@@ -6685,7 +6685,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t xml:space="preserve">KIDS SUN CARE SPF 50+ WET SKIN SPRAY</t>
+          <t xml:space="preserve">Frezyderm Kids Sun Care Spf 50+ Wet Skin Spray</t>
         </is>
       </c>
       <c r="B182">
@@ -6723,7 +6723,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t xml:space="preserve">KIDS SUN CARE SPF 50+ WET SKIN SPRAY</t>
+          <t xml:space="preserve">Frezyderm Kids Sun Care Spf 50+ Wet Skin Spray</t>
         </is>
       </c>
       <c r="B183">
@@ -6761,7 +6761,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t xml:space="preserve">KIDS SUN CARE SPF 50+ WET SKIN SPRAY</t>
+          <t xml:space="preserve">Frezyderm Kids Sun Care Spf 50+ Wet Skin Spray</t>
         </is>
       </c>
       <c r="B184">
@@ -6804,7 +6804,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM KID'S SUN NIP SPF50+ 175ml</t>
+          <t xml:space="preserve">Frezyderm Kid'S Sun Nip Spf50+ 175ml</t>
         </is>
       </c>
       <c r="B185">
@@ -6837,7 +6837,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t xml:space="preserve">LICE FREE SET</t>
+          <t xml:space="preserve">Frezyderm Lice Free Set</t>
         </is>
       </c>
       <c r="B186">
@@ -6875,7 +6875,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t xml:space="preserve">LICE REP EXTREME SPRAY</t>
+          <t xml:space="preserve">Frezyderm Lice Rep Extreme Spray</t>
         </is>
       </c>
       <c r="B187">
@@ -6918,7 +6918,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t xml:space="preserve">LICE REP EXTREME SPRAY</t>
+          <t xml:space="preserve">Frezyderm Lice Rep Extreme Spray</t>
         </is>
       </c>
       <c r="B188">
@@ -6956,7 +6956,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM Lipolysis Cream Booster 5ml</t>
+          <t xml:space="preserve">Frezyderm Lipolysis Cream Booster 5ml</t>
         </is>
       </c>
       <c r="B189">
@@ -6984,7 +6984,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t xml:space="preserve">MACROGOL ADULTS 3350</t>
+          <t xml:space="preserve">Frezyderm Macrogol Adults 3350</t>
         </is>
       </c>
       <c r="B190">
@@ -7022,7 +7022,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t xml:space="preserve">MACROGOL KIDS 3350</t>
+          <t xml:space="preserve">Frezyderm Macrogol Kids 3350</t>
         </is>
       </c>
       <c r="B191">
@@ -7060,7 +7060,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM Matte Effect Cream 50ml</t>
+          <t xml:space="preserve">Frezyderm Matte Effect Cream 50ml</t>
         </is>
       </c>
       <c r="B192">
@@ -7093,7 +7093,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM Mediated Cream-Gel 50ml</t>
+          <t xml:space="preserve">Frezyderm Mediated Cream-Gel 50ml</t>
         </is>
       </c>
       <c r="B193">
@@ -7126,7 +7126,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM MEDIATED SH.DRY DANDR.200ML</t>
+          <t xml:space="preserve">Frezyderm Mediated Sh.Dry Dandr.200Ml</t>
         </is>
       </c>
       <c r="B194">
@@ -7154,7 +7154,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t xml:space="preserve">AC-NORM MICELLAR WATER</t>
+          <t xml:space="preserve">Frezyderm Ac-Norm Micellar Water</t>
         </is>
       </c>
       <c r="B195">
@@ -7192,7 +7192,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM MILD WASH  150ML</t>
+          <t xml:space="preserve">Frezyderm Mild Wash 150Ml</t>
         </is>
       </c>
       <c r="B196">
@@ -7220,7 +7220,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t xml:space="preserve">MILD WASH LIQUID</t>
+          <t xml:space="preserve">Frezyderm Mild Wash Liquid</t>
         </is>
       </c>
       <c r="B197">
@@ -7258,7 +7258,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM MOISTURIZING 24H 20+ 50 ML</t>
+          <t xml:space="preserve">Frezyderm Moisturizing 24H 20+ 50 Ml</t>
         </is>
       </c>
       <c r="B198">
@@ -7291,7 +7291,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM MOISTURIZING PLUS 30+ 50 ML</t>
+          <t xml:space="preserve">Frezyderm Moisturizing Plus 30+ 50 Ml</t>
         </is>
       </c>
       <c r="B199">
@@ -7324,7 +7324,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM Moisturizing Rich Cream 50ml</t>
+          <t xml:space="preserve">Frezyderm Moisturizing Rich Cream 50ml</t>
         </is>
       </c>
       <c r="B200">
@@ -7357,7 +7357,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM MOUTHWASH GINGIVITIS 250ML</t>
+          <t xml:space="preserve">Frezyderm Mouthwash Gingivitis 250Ml</t>
         </is>
       </c>
       <c r="B201">
@@ -7385,7 +7385,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t xml:space="preserve">HOMEOPATHY MOUTHWASH</t>
+          <t xml:space="preserve">Frezyderm Homeopathy Mouthwash</t>
         </is>
       </c>
       <c r="B202">
@@ -7423,7 +7423,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t xml:space="preserve">BLACK &amp;amp; POLISH OXYGEN MOUTHWASH </t>
+          <t xml:space="preserve">Frezyderm Black &amp;amp; Polish Oxygen Mouthwash</t>
         </is>
       </c>
       <c r="B203">
@@ -7461,7 +7461,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM MOUTHWASH PERIODONTITIS 250ML</t>
+          <t xml:space="preserve">Frezyderm Mouthwash Periodontitis 250Ml</t>
         </is>
       </c>
       <c r="B204">
@@ -7489,7 +7489,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t xml:space="preserve">SENSITIVE TEETH MOUTHWASH</t>
+          <t xml:space="preserve">Frezyderm Sensitive Teeth Mouthwash</t>
         </is>
       </c>
       <c r="B205">
@@ -7527,7 +7527,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM NASAL OINTMENT  15ML</t>
+          <t xml:space="preserve">Frezyderm Nasal Ointment 15Ml</t>
         </is>
       </c>
       <c r="B206">
@@ -7560,7 +7560,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t xml:space="preserve">NAZAL CLEANER ALLERGY (0,9% NaCl)</t>
+          <t xml:space="preserve">Frezyderm Nazal Cleaner Allergy (0,9% NaCl)</t>
         </is>
       </c>
       <c r="B207">
@@ -7598,7 +7598,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t xml:space="preserve">NAZAL CLEANER ΙSOTONIC</t>
+          <t xml:space="preserve">Frezyderm Nazal Cleaner ΙSotonic</t>
         </is>
       </c>
       <c r="B208">
@@ -7636,7 +7636,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t xml:space="preserve">NAZAL CLEANER COLD (2,2% NaCl)</t>
+          <t xml:space="preserve">Frezyderm Nazal Cleaner Cold (2,2% NaCl)</t>
         </is>
       </c>
       <c r="B209">
@@ -7674,7 +7674,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t xml:space="preserve">NAZAL CLEANER COLD SPICY (2,2% NaCl) </t>
+          <t xml:space="preserve">Frezyderm Nazal Cleaner Cold Spicy (2,2% NaCl)</t>
         </is>
       </c>
       <c r="B210">
@@ -7712,7 +7712,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t xml:space="preserve">NAZAL CLEANER HOMEO (2,2% NaCl)</t>
+          <t xml:space="preserve">Frezyderm Nazal Cleaner Homeo (2,2% NaCl)</t>
         </is>
       </c>
       <c r="B211">
@@ -7750,7 +7750,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t xml:space="preserve">NAZAL CLEANER MOIST (0,9% NaCl) </t>
+          <t xml:space="preserve">Frezyderm Nazal Cleaner Moist (0,9% NaCl)</t>
         </is>
       </c>
       <c r="B212">
@@ -7788,7 +7788,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t xml:space="preserve">NAZAL CLEANER SINUS PROTECT (0,9% NaCl) </t>
+          <t xml:space="preserve">Frezyderm Nazal Cleaner Sinus Protect (0,9% NaCl)</t>
         </is>
       </c>
       <c r="B213">
@@ -7826,7 +7826,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM Night Force A + E Cream 50ml</t>
+          <t xml:space="preserve">Frezyderm Night Force A + E Cream 50ml</t>
         </is>
       </c>
       <c r="B214">
@@ -7859,7 +7859,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t xml:space="preserve">NIPPLE EMOLLIENT CREAM-GEL </t>
+          <t xml:space="preserve">Frezyderm Nipple Emollient Cream-Gel</t>
         </is>
       </c>
       <c r="B215">
@@ -7902,7 +7902,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM Nipple Care Restructuring Cream-Gel 40ml</t>
+          <t xml:space="preserve">Frezyderm Nipple Care Restructuring Cream-Gel 40ml</t>
         </is>
       </c>
       <c r="B216">
@@ -7935,7 +7935,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t xml:space="preserve">ODOR BLOCKER TOOTHPASTE </t>
+          <t xml:space="preserve">Frezyderm Odor Blocker Toothpaste</t>
         </is>
       </c>
       <c r="B217">
@@ -7973,7 +7973,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t xml:space="preserve">ODOR BLOCKER MOUTHWASH</t>
+          <t xml:space="preserve">Frezyderm Odor Blocker Mouthwash</t>
         </is>
       </c>
       <c r="B218">
@@ -8011,7 +8011,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM ORGANIC CHAMOMILE 15GR</t>
+          <t xml:space="preserve">Frezyderm Organic Chamomile 15Gr</t>
         </is>
       </c>
       <c r="B219">
@@ -8039,7 +8039,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM Organic Fennel 60gr</t>
+          <t xml:space="preserve">Frezyderm Organic Fennel 60gr</t>
         </is>
       </c>
       <c r="B220">
@@ -8072,7 +8072,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM Peptides &amp; Stems Cream Booster 5ml</t>
+          <t xml:space="preserve">Frezyderm Peptides &amp; Stems Cream Booster 5ml</t>
         </is>
       </c>
       <c r="B221">
@@ -8100,7 +8100,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t xml:space="preserve">PLAQUE &amp;amp; TARTAR MOUTHWASH</t>
+          <t xml:space="preserve">Frezyderm Plaque &amp;amp; Tartar Mouthwash</t>
         </is>
       </c>
       <c r="B222">
@@ -8138,7 +8138,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM PRELACTIC OVULES CE 10OLUVES</t>
+          <t xml:space="preserve">Frezyderm Prelactic Ovules Ce 10Oluves</t>
         </is>
       </c>
       <c r="B223">
@@ -8166,7 +8166,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM PRELACTIC VAGINAL CREAM 50ML</t>
+          <t xml:space="preserve">Frezyderm Prelactic Vaginal Cream 50Ml</t>
         </is>
       </c>
       <c r="B224">
@@ -8199,7 +8199,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM PREVENSTRIA CREAM 150ML</t>
+          <t xml:space="preserve">Frezyderm Prevenstria Cream 150Ml</t>
         </is>
       </c>
       <c r="B225">
@@ -8227,7 +8227,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t xml:space="preserve">PREVENSTRIA PROTECTIVE ANTI-STRIA CREAM </t>
+          <t xml:space="preserve">Frezyderm Prevenstria Protective Anti-Stria Cream</t>
         </is>
       </c>
       <c r="B226">
@@ -8265,7 +8265,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM Prodilac Ease 10τμχ</t>
+          <t xml:space="preserve">Frezyderm Prodilac Ease 10τμχ</t>
         </is>
       </c>
       <c r="B227">
@@ -8293,7 +8293,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM PRODILAC EASE 30 STICKS</t>
+          <t xml:space="preserve">Frezyderm Prodilac Ease 30 Sticks</t>
         </is>
       </c>
       <c r="B228">
@@ -8321,7 +8321,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t xml:space="preserve">PRODILAC IMMUNO SHIELD FAST MELT</t>
+          <t xml:space="preserve">Frezyderm Prodilac Immuno Shield Fast Melt</t>
         </is>
       </c>
       <c r="B229">
@@ -8359,7 +8359,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t xml:space="preserve">PRODILAC IMMUNO SHIELD START</t>
+          <t xml:space="preserve">Frezyderm Prodilac Immuno Shield Start</t>
         </is>
       </c>
       <c r="B230">
@@ -8397,7 +8397,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t xml:space="preserve">PRODILAC IMMUNO SHIELD START</t>
+          <t xml:space="preserve">Frezyderm Prodilac Immuno Shield Start</t>
         </is>
       </c>
       <c r="B231">
@@ -8435,7 +8435,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t xml:space="preserve">PRODILAC KIDS</t>
+          <t xml:space="preserve">Frezyderm Prodilac Kids</t>
         </is>
       </c>
       <c r="B232">
@@ -8473,7 +8473,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM PRODILAC ORAL (30 ΜΑΣΩΜΕΝΑ ΔΙΣΚΙΑ)-  (Φ.Π.Α 6%)</t>
+          <t xml:space="preserve">Frezyderm Prodilac Oral (30 ΜΑΣΩΜΕΝΑ ΔΙΣΚΙΑ)- (Φ.Π.Α 6%)</t>
         </is>
       </c>
       <c r="B233">
@@ -8501,7 +8501,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t xml:space="preserve">PRODILAC KIDS</t>
+          <t xml:space="preserve">Frezyderm Prodilac Kids</t>
         </is>
       </c>
       <c r="B234">
@@ -8539,7 +8539,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t xml:space="preserve">PRODILAC RESTORE</t>
+          <t xml:space="preserve">Frezyderm Prodilac Restore</t>
         </is>
       </c>
       <c r="B235">
@@ -8577,7 +8577,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t xml:space="preserve">PRODILAC START</t>
+          <t xml:space="preserve">Frezyderm Prodilac Start</t>
         </is>
       </c>
       <c r="B236">
@@ -8615,7 +8615,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t xml:space="preserve">PRODILAC START</t>
+          <t xml:space="preserve">Frezyderm Prodilac Start</t>
         </is>
       </c>
       <c r="B237">
@@ -8653,7 +8653,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM PROFLAMINE 40ML</t>
+          <t xml:space="preserve">Frezyderm Proflamine 40Ml</t>
         </is>
       </c>
       <c r="B238">
@@ -8686,7 +8686,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t xml:space="preserve">AC-NORM ACTIVE CLEANSER</t>
+          <t xml:space="preserve">Frezyderm Ac-Norm Active Cleanser</t>
         </is>
       </c>
       <c r="B239">
@@ -8724,7 +8724,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t xml:space="preserve">AC-NORM MEDILIKE EFFECT 1 CREAM</t>
+          <t xml:space="preserve">Frezyderm Ac-Norm Medilike Effect 1 Cream</t>
         </is>
       </c>
       <c r="B240">
@@ -8762,7 +8762,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t xml:space="preserve">ANTI-WRINKLE RICH DAY CREAM ΝΕΣΕΣΕΡ ΜΕ ΔΩΡΟ ΔΕΙΓΜΑ ANTI-WRINKLE NIGHT 15ml, EYE CREAM 5ml &amp;amp; VELVET COLORS MEDIUM 2ml</t>
+          <t xml:space="preserve">Frezyderm Anti-Wrinkle Rich Day Cream ΝΕΣΕΣΕΡ ΜΕ ΔΩΡΟ ΔΕΙΓΜΑ Anti-Wrinkle Night 15ml, Eye Cream 5ml &amp;amp; Velvet Colors Medium 2ml</t>
         </is>
       </c>
       <c r="B241">
@@ -8800,7 +8800,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t xml:space="preserve">ANTI-WRINKLE RICH DAY CREAM ΝΕΣΕΣΕΡ ΜΕ ΔΩΡΟ ΔΕΙΓΜΑ ANTI-WRINKLE NIGHT 15ml, EYE CREAM 5ml &amp;amp; VELVET COLORS MEDIUM 2ml</t>
+          <t xml:space="preserve">Frezyderm Anti-Wrinkle Rich Day Cream ΝΕΣΕΣΕΡ ΜΕ ΔΩΡΟ ΔΕΙΓΜΑ Anti-Wrinkle Night 15ml, Eye Cream 5ml &amp;amp; Velvet Colors Medium 2ml</t>
         </is>
       </c>
       <c r="B242">
@@ -8843,7 +8843,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t xml:space="preserve">BABY BATH</t>
+          <t xml:space="preserve">Frezyderm Baby Bath</t>
         </is>
       </c>
       <c r="B243">
@@ -8881,7 +8881,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t xml:space="preserve">BABY SUN CARE SPF 50 100ml ΜΕ ΔΩΡΟ ΕΠΙΠΛΕΟΝ ΠΟΣΟΤΗΤΑ 50ml</t>
+          <t xml:space="preserve">Frezyderm Baby Sun Care Spf 50 100ml ΜΕ ΔΩΡΟ ΕΠΙΠΛΕΟΝ ΠΟΣΟΤΗΤΑ 50ml</t>
         </is>
       </c>
       <c r="B244">
@@ -8919,7 +8919,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t xml:space="preserve">BABY SUN CARE SPF 50 100ml ΜΕ ΔΩΡΟ ΕΠΙΠΛΕΟΝ ΠΟΣΟΤΗΤΑ 50ml</t>
+          <t xml:space="preserve">Frezyderm Baby Sun Care Spf 50 100ml ΜΕ ΔΩΡΟ ΕΠΙΠΛΕΟΝ ΠΟΣΟΤΗΤΑ 50ml</t>
         </is>
       </c>
       <c r="B245">
@@ -8957,7 +8957,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t xml:space="preserve">BABY HYDRA MILK</t>
+          <t xml:space="preserve">Frezyderm Baby Hydra Milk</t>
         </is>
       </c>
       <c r="B246">
@@ -8995,7 +8995,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t xml:space="preserve">BABY HYDRA MILK</t>
+          <t xml:space="preserve">Frezyderm Baby Hydra Milk</t>
         </is>
       </c>
       <c r="B247">
@@ -9038,7 +9038,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t xml:space="preserve">BABY BATH</t>
+          <t xml:space="preserve">Frezyderm Baby Bath</t>
         </is>
       </c>
       <c r="B248">
@@ -9076,7 +9076,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t xml:space="preserve">DERMOFILIA HAND CREAM 75ml ΜΕ ΔΩΡΟ ΕΠΙΠΛΕΟΝ ΠΟΣΟΤΗΤΑ 40ml</t>
+          <t xml:space="preserve">Frezyderm Dermofilia Hand Cream 75ml ΜΕ ΔΩΡΟ ΕΠΙΠΛΕΟΝ ΠΟΣΟΤΗΤΑ 40ml</t>
         </is>
       </c>
       <c r="B249">
@@ -9114,7 +9114,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t xml:space="preserve">HAIR FORCE SHAMPOO MEN</t>
+          <t xml:space="preserve">Frezyderm Hair Force Shampoo Men</t>
         </is>
       </c>
       <c r="B250">
@@ -9152,7 +9152,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t xml:space="preserve">ANTI-WRINKLE RICH DAY CREAM ΝΕΣΕΣΕΡ ΜΕ ΔΩΡΟ ΔΕΙΓΜΑ ANTI-WRINKLE NIGHT 15ml, EYE CREAM 5ml &amp;amp; VELVET COLORS MEDIUM 2ml</t>
+          <t xml:space="preserve">Frezyderm Anti-Wrinkle Rich Day Cream ΝΕΣΕΣΕΡ ΜΕ ΔΩΡΟ ΔΕΙΓΜΑ Anti-Wrinkle Night 15ml, Eye Cream 5ml &amp;amp; Velvet Colors Medium 2ml</t>
         </is>
       </c>
       <c r="B251">
@@ -9190,7 +9190,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t xml:space="preserve">INTIM AREA WIPES</t>
+          <t xml:space="preserve">Frezyderm Intim Area Wipes</t>
         </is>
       </c>
       <c r="B252">
@@ -9228,7 +9228,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t xml:space="preserve">BABY BATH</t>
+          <t xml:space="preserve">Frezyderm Baby Bath</t>
         </is>
       </c>
       <c r="B253">
@@ -9266,7 +9266,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t xml:space="preserve">BABY BATH</t>
+          <t xml:space="preserve">Frezyderm Baby Bath</t>
         </is>
       </c>
       <c r="B254">
@@ -9304,7 +9304,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUN SCREEN VELVET FACE SPF 30 </t>
+          <t xml:space="preserve">Frezyderm Sun Screen Velvet Face Spf 30</t>
         </is>
       </c>
       <c r="B255">
@@ -9342,7 +9342,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t xml:space="preserve">CRILEN ΓΑΛΑΚΤΩΜΑ 125ml ΜΕ ΔΩΡΟ ΕΠΙΠΛΕΟΝ ΠΟΣΟΤΗΤΑ 40ml</t>
+          <t xml:space="preserve">Frezyderm Crilen ΓΑΛΑΚΤΩΜΑ 125ml ΜΕ ΔΩΡΟ ΕΠΙΠΛΕΟΝ ΠΟΣΟΤΗΤΑ 40ml</t>
         </is>
       </c>
       <c r="B256">
@@ -9380,7 +9380,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t xml:space="preserve">LICE REP EXTREME SPRAY</t>
+          <t xml:space="preserve">Frezyderm Lice Rep Extreme Spray</t>
         </is>
       </c>
       <c r="B257">
@@ -9418,7 +9418,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t xml:space="preserve">DE-MAKE UP 4 in 1</t>
+          <t xml:space="preserve">Frezyderm De-Make Up 4 in 1</t>
         </is>
       </c>
       <c r="B258">
@@ -9456,7 +9456,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM Promo Prevenstria Cream για την Προ?ληψη των Ραγα?δων 150ml &amp; ΔΩΡΟ Επιπλέον 100ml</t>
+          <t xml:space="preserve">Frezyderm Promo Prevenstria Cream για την Προ?ληψη των Ραγα?δων 150ml &amp; ΔΩΡΟ Επιπλέον 100ml</t>
         </is>
       </c>
       <c r="B259">
@@ -9494,7 +9494,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t xml:space="preserve">SENSITEETH KIDS TOOTHPASTE 500ppm</t>
+          <t xml:space="preserve">Frezyderm Sensiteeth Kids Toothpaste 500ppm</t>
         </is>
       </c>
       <c r="B260">
@@ -9537,7 +9537,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t xml:space="preserve">SENSITIVE KIDS MAGIC SPRAY</t>
+          <t xml:space="preserve">Frezyderm Sensitive Kids Magic Spray</t>
         </is>
       </c>
       <c r="B261">
@@ -9575,7 +9575,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t xml:space="preserve">SENSITIVE KIDS STYLING GEL</t>
+          <t xml:space="preserve">Frezyderm Sensitive Kids Styling Gel</t>
         </is>
       </c>
       <c r="B262">
@@ -9613,7 +9613,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t xml:space="preserve">ACTIVE SUN SCREEN LIP BALM SPF 50+</t>
+          <t xml:space="preserve">Frezyderm Active Sun Screen Lip Balm Spf 50+</t>
         </is>
       </c>
       <c r="B263">
@@ -9651,7 +9651,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM PROPOLIS SPRAY 30 ML</t>
+          <t xml:space="preserve">Frezyderm Propolis Spray 30 Ml</t>
         </is>
       </c>
       <c r="B264">
@@ -9679,7 +9679,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t xml:space="preserve">PS.T. FLAKES BALANCE CREAM STEP 3</t>
+          <t xml:space="preserve">Frezyderm Ps.T. Flakes Balance Cream Step 3</t>
         </is>
       </c>
       <c r="B265">
@@ -9717,7 +9717,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t xml:space="preserve">PS.T. CLEANSER STEP 1</t>
+          <t xml:space="preserve">Frezyderm Ps.T. Cleanser Step 1</t>
         </is>
       </c>
       <c r="B266">
@@ -9755,7 +9755,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM PS T Keratolytic Cream Step 2  200ml</t>
+          <t xml:space="preserve">Frezyderm Ps T Keratolytic Cream Step 2 200ml</t>
         </is>
       </c>
       <c r="B267">
@@ -9793,7 +9793,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t xml:space="preserve">PS.T. SECOND SKIN CREAM STEP 4</t>
+          <t xml:space="preserve">Frezyderm Ps.T. Second Skin Cream Step 4</t>
         </is>
       </c>
       <c r="B268">
@@ -9831,7 +9831,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t xml:space="preserve">PS.T. SECOND SKIN CREAM STEP 4</t>
+          <t xml:space="preserve">Frezyderm Ps.T. Second Skin Cream Step 4</t>
         </is>
       </c>
       <c r="B269">
@@ -9869,7 +9869,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t xml:space="preserve">FACE SERUM PURE COLLAGEN - Ορός Σύσφιξης Προσώπου με Κολλαγόνο</t>
+          <t xml:space="preserve">Frezyderm Face Serum Pure Collagen - Ορός Σύσφιξης Προσώπου με Κολλαγόνο</t>
         </is>
       </c>
       <c r="B270">
@@ -9907,7 +9907,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM RECONSTRIA 75ML</t>
+          <t xml:space="preserve">Frezyderm Reconstria 75Ml</t>
         </is>
       </c>
       <c r="B271">
@@ -9940,7 +9940,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t xml:space="preserve">RECONSTRIA RESTRUCTURING ANTI-STRIA CREAM</t>
+          <t xml:space="preserve">Frezyderm Reconstria Restructuring Anti-Stria Cream</t>
         </is>
       </c>
       <c r="B272">
@@ -9978,7 +9978,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM RECTANAL AID CREAM 50ML</t>
+          <t xml:space="preserve">Frezyderm Rectanal Aid Cream 50Ml</t>
         </is>
       </c>
       <c r="B273">
@@ -10016,7 +10016,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM Reform Abdomen Care Cream 150ml</t>
+          <t xml:space="preserve">Frezyderm Reform Abdomen Care Cream 150ml</t>
         </is>
       </c>
       <c r="B274">
@@ -10044,7 +10044,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t xml:space="preserve">REVITALIZATION HYDROGEL EYE PATCH</t>
+          <t xml:space="preserve">Frezyderm Revitalization Hydrogel Eye Patch</t>
         </is>
       </c>
       <c r="B275">
@@ -10087,7 +10087,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM Revitalizing Serum 30ml</t>
+          <t xml:space="preserve">Frezyderm Revitalizing Serum 30ml</t>
         </is>
       </c>
       <c r="B276">
@@ -10115,7 +10115,7 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM Rinopure Φυσιολογικός Ορός 30τμχ x 5ml</t>
+          <t xml:space="preserve">Frezyderm Rinopure Φυσιολογικός Ορός 30τμχ x 5ml</t>
         </is>
       </c>
       <c r="B277">
@@ -10148,7 +10148,7 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUN SCREEN ON THE MOVE SPF 50</t>
+          <t xml:space="preserve">Frezyderm Sun Screen On The Move Spf 50</t>
         </is>
       </c>
       <c r="B278">
@@ -10186,7 +10186,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t xml:space="preserve">SEA SIDE DRY MIST SPF 50+</t>
+          <t xml:space="preserve">Frezyderm Sea Side Dry Mist Spf 50+</t>
         </is>
       </c>
       <c r="B279">
@@ -10224,7 +10224,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t xml:space="preserve">SEAWEED HYDROGEL CARE PATCH</t>
+          <t xml:space="preserve">Frezyderm Seaweed Hydrogel Care Patch</t>
         </is>
       </c>
       <c r="B280">
@@ -10262,7 +10262,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t xml:space="preserve">SEB EXCESS SHAMPOO</t>
+          <t xml:space="preserve">Frezyderm Seb Excess Shampoo</t>
         </is>
       </c>
       <c r="B281">
@@ -10300,7 +10300,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t xml:space="preserve">SEB EXCESS SHAMPOO</t>
+          <t xml:space="preserve">Frezyderm Seb Excess Shampoo</t>
         </is>
       </c>
       <c r="B282">
@@ -10338,7 +10338,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t xml:space="preserve">SEBUM CONTROL SHAMPOO</t>
+          <t xml:space="preserve">Frezyderm Sebum Control Shampoo</t>
         </is>
       </c>
       <c r="B283">
@@ -10376,7 +10376,7 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t xml:space="preserve">SEBUM CONTROL SHAMPOO</t>
+          <t xml:space="preserve">Frezyderm Sebum Control Shampoo</t>
         </is>
       </c>
       <c r="B284">
@@ -10414,7 +10414,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM Self Care Gel 75ml</t>
+          <t xml:space="preserve">Frezyderm Self Care Gel 75ml</t>
         </is>
       </c>
       <c r="B285">
@@ -10452,7 +10452,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t xml:space="preserve">SELF CARE GEL INTIM LUBRICANT CARE</t>
+          <t xml:space="preserve">Frezyderm Self Care Gel Intim Lubricant Care</t>
         </is>
       </c>
       <c r="B286">
@@ -10490,7 +10490,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t xml:space="preserve">SELF TAN BODY SHAPE</t>
+          <t xml:space="preserve">Frezyderm Self Tan Body Shape</t>
         </is>
       </c>
       <c r="B287">
@@ -10528,7 +10528,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM SENSI KID'S B.MILK+FAMILY200ml</t>
+          <t xml:space="preserve">Frezyderm Sensi Kid'S B.Milk+Family200ml</t>
         </is>
       </c>
       <c r="B288">
@@ -10556,7 +10556,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM SENSI KID'S HAIR STYLING GEL 100ml</t>
+          <t xml:space="preserve">Frezyderm Sensi Kid'S Hair Styling Gel 100ml</t>
         </is>
       </c>
       <c r="B289">
@@ -10589,7 +10589,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t xml:space="preserve">SENSITEETH EPISMALTO TOOTHPASTE 1.450ppm</t>
+          <t xml:space="preserve">Frezyderm Sensiteeth Epismalto Toothpaste 1.450ppm</t>
         </is>
       </c>
       <c r="B290">
@@ -10627,7 +10627,7 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t xml:space="preserve">SENSITEETH FIRST TOOTHPASTE </t>
+          <t xml:space="preserve">Frezyderm Sensiteeth First Toothpaste</t>
         </is>
       </c>
       <c r="B291">
@@ -10665,7 +10665,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t xml:space="preserve">SENSITEETH KIDS APHTHAE GEL</t>
+          <t xml:space="preserve">Frezyderm Sensiteeth Kids Aphthae Gel</t>
         </is>
       </c>
       <c r="B292">
@@ -10703,7 +10703,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t xml:space="preserve">SENSITEETH KIDS MOUTHWASH </t>
+          <t xml:space="preserve">Frezyderm Sensiteeth Kids Mouthwash</t>
         </is>
       </c>
       <c r="B293">
@@ -10741,7 +10741,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t xml:space="preserve">SENSITEETH KIDS MOUTHWASH </t>
+          <t xml:space="preserve">Frezyderm Sensiteeth Kids Mouthwash</t>
         </is>
       </c>
       <c r="B294">
@@ -10784,7 +10784,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t xml:space="preserve">SENSITEETH KIDS TOOTHPASTE 500ppm</t>
+          <t xml:space="preserve">Frezyderm Sensiteeth Kids Toothpaste 500ppm</t>
         </is>
       </c>
       <c r="B295">
@@ -10822,7 +10822,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t xml:space="preserve">SENSITEETH FIRST TOOTHPASTE </t>
+          <t xml:space="preserve">Frezyderm Sensiteeth First Toothpaste</t>
         </is>
       </c>
       <c r="B296">
@@ -10860,7 +10860,7 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t xml:space="preserve">SENSITIVE KIDS INTIM GIRL FOAM</t>
+          <t xml:space="preserve">Frezyderm Sensitive Kids Intim Girl Foam</t>
         </is>
       </c>
       <c r="B297">
@@ -10898,7 +10898,7 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t xml:space="preserve">SENSITIVE KIDS SHAMPOO GIRLS</t>
+          <t xml:space="preserve">Frezyderm Sensitive Kids Shampoo Girls</t>
         </is>
       </c>
       <c r="B298">
@@ -10936,7 +10936,7 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t xml:space="preserve">SENSITIVE KIDS SHAMPOO BOYS</t>
+          <t xml:space="preserve">Frezyderm Sensitive Kids Shampoo Boys</t>
         </is>
       </c>
       <c r="B299">
@@ -10974,7 +10974,7 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t xml:space="preserve">SENSITIVE KIDS INTIM GIRL FOAM</t>
+          <t xml:space="preserve">Frezyderm Sensitive Kids Intim Girl Foam</t>
         </is>
       </c>
       <c r="B300">
@@ -11012,7 +11012,7 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t xml:space="preserve">SENSITIVE KIDS SHOWER BATH</t>
+          <t xml:space="preserve">Frezyderm Sensitive Kids Shower Bath</t>
         </is>
       </c>
       <c r="B301">
@@ -11050,7 +11050,7 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t xml:space="preserve">SENSITIVE RED SKIN FACIAL CREAM</t>
+          <t xml:space="preserve">Frezyderm Sensitive Red Skin Facial Cream</t>
         </is>
       </c>
       <c r="B302">
@@ -11093,7 +11093,7 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t xml:space="preserve">SENSITIVE RED SKIN TINTED SPF 30 CREAM</t>
+          <t xml:space="preserve">Frezyderm Sensitive Red Skin Tinted Spf 30 Cream</t>
         </is>
       </c>
       <c r="B303">
@@ -11131,7 +11131,7 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t xml:space="preserve">SKIN CLEANSER</t>
+          <t xml:space="preserve">Frezyderm Skin Cleanser</t>
         </is>
       </c>
       <c r="B304">
@@ -11169,7 +11169,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t xml:space="preserve">FACE SERUM SUPER SKIN CODE - Αντιρυτιδικός Ορός </t>
+          <t xml:space="preserve">Frezyderm Face Serum Super Skin Code - Αντιρυτιδικός Ορός</t>
         </is>
       </c>
       <c r="B305">
@@ -11207,7 +11207,7 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM Skin Nursery Vitamin B Cream Booster 5ml</t>
+          <t xml:space="preserve">Frezyderm Skin Nursery Vitamin B Cream Booster 5ml</t>
         </is>
       </c>
       <c r="B306">
@@ -11235,7 +11235,7 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM Skin Radiance Cream Booster 5ml</t>
+          <t xml:space="preserve">Frezyderm Skin Radiance Cream Booster 5ml</t>
         </is>
       </c>
       <c r="B307">
@@ -11263,7 +11263,7 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM Skin Restart Vitamin A Cream Booster 5ml</t>
+          <t xml:space="preserve">Frezyderm Skin Restart Vitamin A Cream Booster 5ml</t>
         </is>
       </c>
       <c r="B308">
@@ -11291,7 +11291,7 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t xml:space="preserve">SOOTH BALM</t>
+          <t xml:space="preserve">Frezyderm Sooth Balm</t>
         </is>
       </c>
       <c r="B309">
@@ -11334,7 +11334,7 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t xml:space="preserve">SPOT END CORRECTIVE</t>
+          <t xml:space="preserve">Frezyderm Spot End Corrective</t>
         </is>
       </c>
       <c r="B310">
@@ -11372,7 +11372,7 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t xml:space="preserve">SPOT END DAY CREAM SPF 15</t>
+          <t xml:space="preserve">Frezyderm Spot End Day Cream Spf 15</t>
         </is>
       </c>
       <c r="B311">
@@ -11410,7 +11410,7 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t xml:space="preserve">SPOT END ESSENCE ACTIVE GEL</t>
+          <t xml:space="preserve">Frezyderm Spot End Essence Active Gel</t>
         </is>
       </c>
       <c r="B312">
@@ -11448,7 +11448,7 @@
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t xml:space="preserve">SPOT END DAY CREAM SPF 15</t>
+          <t xml:space="preserve">Frezyderm Spot End Day Cream Spf 15</t>
         </is>
       </c>
       <c r="B313">
@@ -11486,7 +11486,7 @@
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t xml:space="preserve">SPOT END DAY CREAM SPF 15</t>
+          <t xml:space="preserve">Frezyderm Spot End Day Cream Spf 15</t>
         </is>
       </c>
       <c r="B314">
@@ -11524,7 +11524,7 @@
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t xml:space="preserve">KIDS SUN CARE SPF 50+ WET SKIN SPRAY</t>
+          <t xml:space="preserve">Frezyderm Kids Sun Care Spf 50+ Wet Skin Spray</t>
         </is>
       </c>
       <c r="B315">
@@ -11562,7 +11562,7 @@
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUN SCREEN ANTI-SEB SPRAY SPF 30</t>
+          <t xml:space="preserve">Frezyderm Sun Screen Anti-Seb Spray Spf 30</t>
         </is>
       </c>
       <c r="B316">
@@ -11600,7 +11600,7 @@
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t xml:space="preserve">ACTIVE SUN SCREEN FACE FOUNDATION SPF 30</t>
+          <t xml:space="preserve">Frezyderm Active Sun Screen Face Foundation Spf 30</t>
         </is>
       </c>
       <c r="B317">
@@ -11638,7 +11638,7 @@
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUN SCREEN VELVET FACE SPF 30 </t>
+          <t xml:space="preserve">Frezyderm Sun Screen Velvet Face Spf 30</t>
         </is>
       </c>
       <c r="B318">
@@ -11676,7 +11676,7 @@
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUN SCREEN CREAM-TO-POWDER SPF 50+</t>
+          <t xml:space="preserve">Frezyderm Sun Screen Cream-To-Powder Spf 50+</t>
         </is>
       </c>
       <c r="B319">
@@ -11714,7 +11714,7 @@
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUN SCREEN INVISIBLE SPRAY SPF 50+ </t>
+          <t xml:space="preserve">Frezyderm Sun Screen Invisible Spray Spf 50+</t>
         </is>
       </c>
       <c r="B320">
@@ -11752,7 +11752,7 @@
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUN SCREEN MOUSSE SPF 50+</t>
+          <t xml:space="preserve">Frezyderm Sun Screen Mousse Spf 50+</t>
         </is>
       </c>
       <c r="B321">
@@ -11790,7 +11790,7 @@
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUN SCREEN MOUSSE SPF 30</t>
+          <t xml:space="preserve">Frezyderm Sun Screen Mousse Spf 30</t>
         </is>
       </c>
       <c r="B322">
@@ -11828,7 +11828,7 @@
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUN SCREEN MOUSSE SPF 30</t>
+          <t xml:space="preserve">Frezyderm Sun Screen Mousse Spf 30</t>
         </is>
       </c>
       <c r="B323">
@@ -11866,7 +11866,7 @@
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUN SCREEN VELVET FACE SPF 30 </t>
+          <t xml:space="preserve">Frezyderm Sun Screen Velvet Face Spf 30</t>
         </is>
       </c>
       <c r="B324">
@@ -11904,7 +11904,7 @@
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUN SCREEN VELVET FACE SPF 50+</t>
+          <t xml:space="preserve">Frezyderm Sun Screen Velvet Face Spf 50+</t>
         </is>
       </c>
       <c r="B325">
@@ -11942,7 +11942,7 @@
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUN SCREEN TAN ACCELERATOR SPF 10</t>
+          <t xml:space="preserve">Frezyderm Sun Screen Tan Accelerator Spf 10</t>
         </is>
       </c>
       <c r="B326">
@@ -11980,7 +11980,7 @@
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUN SCREEN VELVET FACE SPF 50+</t>
+          <t xml:space="preserve">Frezyderm Sun Screen Velvet Face Spf 50+</t>
         </is>
       </c>
       <c r="B327">
@@ -12018,7 +12018,7 @@
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUN SCREEN COLOR VELVET FACE SPF 50+</t>
+          <t xml:space="preserve">Frezyderm Sun Screen Color Velvet Face Spf 50+</t>
         </is>
       </c>
       <c r="B328">
@@ -12056,7 +12056,7 @@
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUN SCREEN COLOR VELVET FACE SPF 50+</t>
+          <t xml:space="preserve">Frezyderm Sun Screen Color Velvet Face Spf 50+</t>
         </is>
       </c>
       <c r="B329">
@@ -12094,7 +12094,7 @@
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUN SCREEN FLUID-TO-POWDER SPF 50+</t>
+          <t xml:space="preserve">Frezyderm Sun Screen Fluid-To-Powder Spf 50+</t>
         </is>
       </c>
       <c r="B330">
@@ -12132,7 +12132,7 @@
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t xml:space="preserve">BLACK &amp; POLISH TOOTHPASTE</t>
+          <t xml:space="preserve">Frezyderm Black &amp; Polish Toothpaste</t>
         </is>
       </c>
       <c r="B331">
@@ -12170,7 +12170,7 @@
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM TOOTHPASTE GINGIVITIS 75ML</t>
+          <t xml:space="preserve">Frezyderm Toothpaste Gingivitis 75Ml</t>
         </is>
       </c>
       <c r="B332">
@@ -12203,7 +12203,7 @@
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t xml:space="preserve">HOMEOPATHY TOOTHPASTE</t>
+          <t xml:space="preserve">Frezyderm Homeopathy Toothpaste</t>
         </is>
       </c>
       <c r="B333">
@@ -12241,7 +12241,7 @@
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t xml:space="preserve">ODOR BLOCKER TOOTHPASTE </t>
+          <t xml:space="preserve">Frezyderm Odor Blocker Toothpaste</t>
         </is>
       </c>
       <c r="B334">
@@ -12279,7 +12279,7 @@
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM TOOTHPASTE PERIODONTITIS 75ML</t>
+          <t xml:space="preserve">Frezyderm Toothpaste Periodontitis 75Ml</t>
         </is>
       </c>
       <c r="B335">
@@ -12312,7 +12312,7 @@
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t xml:space="preserve">PLAQUE &amp;amp; TARTAR TOOTHPASTE</t>
+          <t xml:space="preserve">Frezyderm Plaque &amp;amp; Tartar Toothpaste</t>
         </is>
       </c>
       <c r="B336">
@@ -12350,7 +12350,7 @@
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM TOOTHPASTE PREGNACY 75ML</t>
+          <t xml:space="preserve">Frezyderm Toothpaste Pregnacy 75Ml</t>
         </is>
       </c>
       <c r="B337">
@@ -12383,7 +12383,7 @@
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t xml:space="preserve">SENSITIVE TEETH TOOTHPASTE</t>
+          <t xml:space="preserve">Frezyderm Sensitive Teeth Toothpaste</t>
         </is>
       </c>
       <c r="B338">
@@ -12421,7 +12421,7 @@
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t xml:space="preserve">WHITENING TOOTHPASTE</t>
+          <t xml:space="preserve">Frezyderm Whitening Toothpaste</t>
         </is>
       </c>
       <c r="B339">
@@ -12459,7 +12459,7 @@
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t xml:space="preserve">INSTANT WHITENING BLUE TOOTHPASTE</t>
+          <t xml:space="preserve">Frezyderm Instant Whitening Blue Toothpaste</t>
         </is>
       </c>
       <c r="B340">
@@ -12497,7 +12497,7 @@
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM Tripleffect Cream Gel 150ml</t>
+          <t xml:space="preserve">Frezyderm Tripleffect Cream Gel 150ml</t>
         </is>
       </c>
       <c r="B341">
@@ -12525,7 +12525,7 @@
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t xml:space="preserve">VELVET STARS SUN SCREEN SPF 50+ </t>
+          <t xml:space="preserve">Frezyderm Velvet Stars Sun Screen Spf 50+</t>
         </is>
       </c>
       <c r="B342">
@@ -12568,7 +12568,7 @@
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t xml:space="preserve">VITAMIN D3</t>
+          <t xml:space="preserve">Frezyderm Vitamin D3</t>
         </is>
       </c>
       <c r="B343">
@@ -12606,7 +12606,7 @@
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t xml:space="preserve">VOLPADERM AHA MILK</t>
+          <t xml:space="preserve">Frezyderm Volpaderm Aha Milk</t>
         </is>
       </c>
       <c r="B344">
@@ -12644,7 +12644,7 @@
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t xml:space="preserve">VOLPADERM AHA CREAM</t>
+          <t xml:space="preserve">Frezyderm Volpaderm Aha Cream</t>
         </is>
       </c>
       <c r="B345">
@@ -12682,7 +12682,7 @@
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t xml:space="preserve">VOLPADERM NAILS TREATING GEL</t>
+          <t xml:space="preserve">Frezyderm Volpaderm Nails Treating Gel</t>
         </is>
       </c>
       <c r="B346">
@@ -12720,7 +12720,7 @@
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM VOMIFREE BOX OF 30 CH TABS1 GR</t>
+          <t xml:space="preserve">Frezyderm Vomifree Box Of 30 Ch Tabs1 Gr</t>
         </is>
       </c>
       <c r="B347">
@@ -12753,7 +12753,7 @@
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t xml:space="preserve">FACE SERUM WRINKLE PLUMPER - Ορός Αντιγήρανσης προσώπου</t>
+          <t xml:space="preserve">Frezyderm Face Serum Wrinkle Plumper - Ορός Αντιγήρανσης προσώπου</t>
         </is>
       </c>
       <c r="B348">
@@ -12791,7 +12791,7 @@
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t xml:space="preserve">FREZYDERM Βιολογικό Χαμομήλι 30gr</t>
+          <t xml:space="preserve">Frezyderm Βιολογικό Χαμομήλι 30gr</t>
         </is>
       </c>
       <c r="B349">

</xml_diff>